<commit_message>
changed rule YAML and test data
</commit_message>
<xml_diff>
--- a/rules/CORE-000929/positive/01/data/unit-test-coreid-CG0001-positive.xlsx
+++ b/rules/CORE-000929/positive/01/data/unit-test-coreid-CG0001-positive.xlsx
@@ -2,9 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="30240" yWindow="-7000" windowWidth="51200" windowHeight="28800" tabRatio="600" firstSheet="0" activeTab="4" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Library" sheetId="1" state="visible" r:id="rId1"/>
@@ -15,15 +14,14 @@
     <sheet name="fa.xpt" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
-    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="5">
     <font>
@@ -34,7 +32,10 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Calibri"/>
+      <family val="2"/>
       <b val="1"/>
+      <sz val="11"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -43,7 +44,10 @@
       <sz val="11"/>
     </font>
     <font>
+      <name val="Calibri"/>
+      <family val="2"/>
       <i val="1"/>
+      <sz val="11"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -52,7 +56,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
@@ -61,13 +65,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFFFCC"/>
-        <bgColor rgb="00FFFFCC"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor rgb="FFFFFFCC"/>
       </patternFill>
     </fill>
   </fills>
@@ -189,9 +188,6 @@
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="1" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
@@ -201,21 +197,24 @@
     <xf numFmtId="3" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="3" fontId="2" fillId="3" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="3" fontId="2" fillId="3" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="3" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -579,7 +578,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:B3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -613,7 +612,7 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>2020-12-18</t>
+          <t>2025-03-28</t>
         </is>
       </c>
     </row>
@@ -629,7 +628,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:B5"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -703,9 +702,9 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:Y7"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="32" customHeight="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
           <t>STUDYID</t>
@@ -791,7 +790,7 @@
           <t>ZBNRIND</t>
         </is>
       </c>
-      <c r="R1" s="7" t="inlineStr">
+      <c r="R1" s="22" t="inlineStr">
         <is>
           <t>ZBSTAT</t>
         </is>
@@ -832,7 +831,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
+    <row r="2" ht="96" customHeight="1">
       <c r="A2" s="9" t="inlineStr">
         <is>
           <t>Study Identifier</t>
@@ -959,7 +958,7 @@
         </is>
       </c>
     </row>
-    <row r="3">
+    <row r="3" ht="16" customHeight="1">
       <c r="A3" s="9" t="inlineStr">
         <is>
           <t>Char</t>
@@ -1163,7 +1162,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" ht="32" customHeight="1">
       <c r="A5" s="13" t="inlineStr">
         <is>
           <t>CDISCPILOT01</t>
@@ -1270,7 +1269,7 @@
         <v>-7</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" ht="48" customHeight="1">
       <c r="A6" s="13" t="inlineStr">
         <is>
           <t>CDISCPILOT01</t>
@@ -1373,7 +1372,7 @@
         <v>-7</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" ht="32" customHeight="1">
       <c r="A7" s="13" t="inlineStr">
         <is>
           <t>CDISCPILOT01</t>
@@ -1490,9 +1489,9 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:U38"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="32" customHeight="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
           <t>STUDYID</t>
@@ -1599,7 +1598,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
+    <row r="2" ht="96" customHeight="1">
       <c r="A2" s="9" t="inlineStr">
         <is>
           <t>Study Identifier</t>
@@ -1706,7 +1705,7 @@
         </is>
       </c>
     </row>
-    <row r="3">
+    <row r="3" ht="16" customHeight="1">
       <c r="A3" s="9" t="inlineStr">
         <is>
           <t>Char</t>
@@ -1878,7 +1877,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" ht="48" customHeight="1">
       <c r="A5" s="13" t="inlineStr">
         <is>
           <t>CDISCPILOT01</t>
@@ -1957,7 +1956,7 @@
         <v>-7</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" ht="48" customHeight="1">
       <c r="A6" s="13" t="inlineStr">
         <is>
           <t>CDISCPILOT01</t>
@@ -2036,7 +2035,7 @@
         <v>-2</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" ht="48" customHeight="1">
       <c r="A7" s="13" t="inlineStr">
         <is>
           <t>CDISCPILOT01</t>
@@ -2119,7 +2118,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" ht="48" customHeight="1">
       <c r="A8" s="13" t="inlineStr">
         <is>
           <t>CDISCPILOT01</t>
@@ -2198,7 +2197,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" ht="48" customHeight="1">
       <c r="A9" s="13" t="inlineStr">
         <is>
           <t>CDISCPILOT01</t>
@@ -2277,7 +2276,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" ht="48" customHeight="1">
       <c r="A10" s="13" t="inlineStr">
         <is>
           <t>CDISCPILOT01</t>
@@ -2358,7 +2357,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="11">
+    <row r="11" ht="48" customHeight="1">
       <c r="A11" s="13" t="inlineStr">
         <is>
           <t>CDISCPILOT01</t>
@@ -2439,7 +2438,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="12">
+    <row r="12" ht="48" customHeight="1">
       <c r="A12" s="13" t="inlineStr">
         <is>
           <t>CDISCPILOT01</t>
@@ -2520,7 +2519,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="13">
+    <row r="13" ht="48" customHeight="1">
       <c r="A13" s="13" t="inlineStr">
         <is>
           <t>CDISCPILOT01</t>
@@ -2601,7 +2600,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="14">
+    <row r="14" ht="32" customHeight="1">
       <c r="A14" s="13" t="inlineStr">
         <is>
           <t>CDISCPILOT01</t>
@@ -2680,7 +2679,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="15">
+    <row r="15" ht="32" customHeight="1">
       <c r="A15" s="13" t="inlineStr">
         <is>
           <t>CDISCPILOT01</t>
@@ -2761,7 +2760,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="16">
+    <row r="16" ht="32" customHeight="1">
       <c r="A16" s="13" t="inlineStr">
         <is>
           <t>CDISCPILOT01</t>
@@ -2842,7 +2841,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="17">
+    <row r="17" ht="32" customHeight="1">
       <c r="A17" s="13" t="inlineStr">
         <is>
           <t>CDISCPILOT01</t>
@@ -2923,7 +2922,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="18">
+    <row r="18" ht="32" customHeight="1">
       <c r="A18" s="13" t="inlineStr">
         <is>
           <t>CDISCPILOT01</t>
@@ -3004,7 +3003,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="19">
+    <row r="19" ht="32" customHeight="1">
       <c r="A19" s="13" t="inlineStr">
         <is>
           <t>CDISCPILOT01</t>
@@ -3085,7 +3084,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="20">
+    <row r="20" ht="32" customHeight="1">
       <c r="A20" s="13" t="inlineStr">
         <is>
           <t>CDISCPILOT01</t>
@@ -3166,7 +3165,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="21">
+    <row r="21" ht="80" customHeight="1">
       <c r="A21" s="13" t="inlineStr">
         <is>
           <t>CDISCPILOT01</t>
@@ -3247,7 +3246,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="22">
+    <row r="22" ht="80" customHeight="1">
       <c r="A22" s="13" t="inlineStr">
         <is>
           <t>CDISCPILOT01</t>
@@ -3328,7 +3327,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="23">
+    <row r="23" ht="80" customHeight="1">
       <c r="A23" s="13" t="inlineStr">
         <is>
           <t>CDISCPILOT01</t>
@@ -3409,7 +3408,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="24">
+    <row r="24" ht="48" customHeight="1">
       <c r="A24" s="13" t="inlineStr">
         <is>
           <t>CDISCPILOT01</t>
@@ -3488,7 +3487,7 @@
         <v>-7</v>
       </c>
     </row>
-    <row r="25">
+    <row r="25" ht="48" customHeight="1">
       <c r="A25" s="13" t="inlineStr">
         <is>
           <t>CDISCPILOT01</t>
@@ -3567,7 +3566,7 @@
         <v>-2</v>
       </c>
     </row>
-    <row r="26">
+    <row r="26" ht="48" customHeight="1">
       <c r="A26" s="13" t="inlineStr">
         <is>
           <t>CDISCPILOT01</t>
@@ -3650,7 +3649,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27">
+    <row r="27" ht="32" customHeight="1">
       <c r="A27" s="13" t="inlineStr">
         <is>
           <t>CDISCPILOT01</t>
@@ -3739,7 +3738,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28">
+    <row r="28" ht="32" customHeight="1">
       <c r="A28" s="13" t="inlineStr">
         <is>
           <t>CDISCPILOT01</t>
@@ -3824,7 +3823,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="29">
+    <row r="29" ht="32" customHeight="1">
       <c r="A29" s="13" t="inlineStr">
         <is>
           <t>CDISCPILOT01</t>
@@ -3909,7 +3908,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="30">
+    <row r="30" ht="32" customHeight="1">
       <c r="A30" s="13" t="inlineStr">
         <is>
           <t>CDISCPILOT01</t>
@@ -3994,7 +3993,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="31">
+    <row r="31" ht="32" customHeight="1">
       <c r="A31" s="13" t="inlineStr">
         <is>
           <t>CDISCPILOT01</t>
@@ -4079,7 +4078,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="32">
+    <row r="32" ht="80" customHeight="1">
       <c r="A32" s="13" t="inlineStr">
         <is>
           <t>CDISCPILOT01</t>
@@ -4164,7 +4163,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="33">
+    <row r="33" ht="32" customHeight="1">
       <c r="A33" s="13" t="inlineStr">
         <is>
           <t>CDISCPILOT01</t>
@@ -4245,7 +4244,7 @@
         <v>-7</v>
       </c>
     </row>
-    <row r="34">
+    <row r="34" ht="32" customHeight="1">
       <c r="A34" s="13" t="inlineStr">
         <is>
           <t>CDISCPILOT01</t>
@@ -4330,7 +4329,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="35">
+    <row r="35" ht="32" customHeight="1">
       <c r="A35" s="13" t="inlineStr">
         <is>
           <t>CDISCPILOT01</t>
@@ -4411,7 +4410,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="36">
+    <row r="36" ht="32" customHeight="1">
       <c r="A36" s="13" t="inlineStr">
         <is>
           <t>CDISCPILOT01</t>
@@ -4492,7 +4491,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="37">
+    <row r="37" ht="32" customHeight="1">
       <c r="A37" s="13" t="inlineStr">
         <is>
           <t>CDISCPILOT01</t>
@@ -4573,7 +4572,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="38">
+    <row r="38" ht="32" customHeight="1">
       <c r="A38" s="13" t="inlineStr">
         <is>
           <t>CDISCPILOT01</t>
@@ -4666,66 +4665,69 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:K8"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="10" max="11"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="7" t="inlineStr">
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="22" t="inlineStr">
         <is>
           <t>STUDYID</t>
         </is>
       </c>
-      <c r="B1" s="7" t="inlineStr">
+      <c r="B1" s="22" t="inlineStr">
         <is>
           <t>DOMAIN</t>
         </is>
       </c>
-      <c r="C1" s="7" t="inlineStr">
+      <c r="C1" s="22" t="inlineStr">
         <is>
           <t>USUBJID</t>
         </is>
       </c>
-      <c r="D1" s="7" t="inlineStr">
+      <c r="D1" s="22" t="inlineStr">
         <is>
           <t>CMSEQ</t>
         </is>
       </c>
-      <c r="E1" s="7" t="inlineStr">
+      <c r="E1" s="22" t="inlineStr">
         <is>
           <t>CMTRT</t>
         </is>
       </c>
-      <c r="F1" s="17" t="inlineStr">
+      <c r="F1" s="22" t="inlineStr">
         <is>
           <t>CMDOSE</t>
         </is>
       </c>
-      <c r="G1" s="17" t="inlineStr">
+      <c r="G1" s="22" t="inlineStr">
         <is>
           <t>CMDOSTXT</t>
         </is>
       </c>
-      <c r="H1" s="7" t="inlineStr">
+      <c r="H1" s="22" t="inlineStr">
         <is>
           <t>CMDOSU</t>
         </is>
       </c>
-      <c r="I1" s="7" t="inlineStr">
+      <c r="I1" s="22" t="inlineStr">
         <is>
           <t>CMDOSFRQ</t>
         </is>
       </c>
-      <c r="J1" s="18" t="inlineStr">
+      <c r="J1" s="17" t="inlineStr">
         <is>
           <t>CMSTDTC</t>
         </is>
       </c>
-      <c r="K1" s="18" t="inlineStr">
+      <c r="K1" s="17" t="inlineStr">
         <is>
           <t>CMENDTC</t>
         </is>
       </c>
     </row>
-    <row r="2">
+    <row r="2" ht="80" customHeight="1">
       <c r="A2" s="11" t="inlineStr">
         <is>
           <t>Study Identifier</t>
@@ -4771,18 +4773,18 @@
           <t>Dosing Frequency per Interval</t>
         </is>
       </c>
-      <c r="J2" s="19" t="inlineStr">
+      <c r="J2" s="18" t="inlineStr">
         <is>
           <t>Start Date/Time of Medication</t>
         </is>
       </c>
-      <c r="K2" s="19" t="inlineStr">
+      <c r="K2" s="18" t="inlineStr">
         <is>
           <t>End Date/Time of Medication</t>
         </is>
       </c>
     </row>
-    <row r="3">
+    <row r="3" ht="16" customHeight="1">
       <c r="A3" s="11" t="inlineStr">
         <is>
           <t>Char</t>
@@ -4828,12 +4830,12 @@
           <t>Char</t>
         </is>
       </c>
-      <c r="J3" s="19" t="inlineStr">
+      <c r="J3" s="18" t="inlineStr">
         <is>
           <t>Char</t>
         </is>
       </c>
-      <c r="K3" s="19" t="inlineStr">
+      <c r="K3" s="18" t="inlineStr">
         <is>
           <t>Char</t>
         </is>
@@ -4874,7 +4876,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" ht="16" customHeight="1">
       <c r="A5" s="16" t="inlineStr">
         <is>
           <t>ABC</t>
@@ -4890,7 +4892,7 @@
           <t>ABC-0002</t>
         </is>
       </c>
-      <c r="D5" s="20" t="n">
+      <c r="D5" s="19" t="n">
         <v>1</v>
       </c>
       <c r="E5" s="16" t="inlineStr">
@@ -4898,8 +4900,8 @@
           <t>ASPIRIN</t>
         </is>
       </c>
-      <c r="F5" s="21" t="n"/>
-      <c r="G5" s="22" t="n">
+      <c r="F5" s="23" t="n"/>
+      <c r="G5" s="24" t="n">
         <v>100</v>
       </c>
       <c r="H5" s="16" t="inlineStr">
@@ -4912,14 +4914,14 @@
           <t>QD</t>
         </is>
       </c>
-      <c r="J5" s="23" t="n">
+      <c r="J5" s="20" t="n">
         <v>37987</v>
       </c>
-      <c r="K5" s="23" t="n">
+      <c r="K5" s="20" t="n">
         <v>37989</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" ht="16" customHeight="1">
       <c r="A6" s="16" t="inlineStr">
         <is>
           <t>ABC</t>
@@ -4935,7 +4937,7 @@
           <t>ABC-0002</t>
         </is>
       </c>
-      <c r="D6" s="20" t="n">
+      <c r="D6" s="19" t="n">
         <v>2</v>
       </c>
       <c r="E6" s="16" t="inlineStr">
@@ -4943,8 +4945,8 @@
           <t>ASPIRIN</t>
         </is>
       </c>
-      <c r="F6" s="21" t="n"/>
-      <c r="G6" s="22" t="n">
+      <c r="F6" s="23" t="n"/>
+      <c r="G6" s="24" t="n">
         <v>100</v>
       </c>
       <c r="H6" s="16" t="inlineStr">
@@ -4957,14 +4959,14 @@
           <t>BID</t>
         </is>
       </c>
-      <c r="J6" s="23" t="n">
+      <c r="J6" s="20" t="n">
         <v>37993</v>
       </c>
-      <c r="K6" s="23" t="n">
+      <c r="K6" s="20" t="n">
         <v>37993</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" ht="16" customHeight="1">
       <c r="A7" s="16" t="inlineStr">
         <is>
           <t>ABC</t>
@@ -4980,7 +4982,7 @@
           <t>ABC-0002</t>
         </is>
       </c>
-      <c r="D7" s="20" t="n">
+      <c r="D7" s="19" t="n">
         <v>3</v>
       </c>
       <c r="E7" s="16" t="inlineStr">
@@ -4988,8 +4990,8 @@
           <t>ASPIRIN</t>
         </is>
       </c>
-      <c r="F7" s="21" t="n"/>
-      <c r="G7" s="22" t="n">
+      <c r="F7" s="23" t="n"/>
+      <c r="G7" s="24" t="n">
         <v>100</v>
       </c>
       <c r="H7" s="16" t="inlineStr">
@@ -5002,14 +5004,14 @@
           <t>QD</t>
         </is>
       </c>
-      <c r="J7" s="23" t="n">
+      <c r="J7" s="20" t="n">
         <v>37995</v>
       </c>
-      <c r="K7" s="23" t="n">
+      <c r="K7" s="20" t="n">
         <v>37995</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" ht="16" customHeight="1">
       <c r="A8" s="16" t="inlineStr">
         <is>
           <t>ABC</t>
@@ -5025,7 +5027,7 @@
           <t>ABC-0003</t>
         </is>
       </c>
-      <c r="D8" s="20" t="n">
+      <c r="D8" s="19" t="n">
         <v>1</v>
       </c>
       <c r="E8" s="16" t="inlineStr">
@@ -5033,8 +5035,8 @@
           <t>ASPIRIN</t>
         </is>
       </c>
-      <c r="F8" s="21" t="n"/>
-      <c r="G8" s="22" t="n">
+      <c r="F8" s="23" t="n"/>
+      <c r="G8" s="24" t="n">
         <v>100</v>
       </c>
       <c r="H8" s="16" t="inlineStr">
@@ -5047,10 +5049,10 @@
           <t>PRN</t>
         </is>
       </c>
-      <c r="J8" s="23" t="n">
+      <c r="J8" s="20" t="n">
         <v>37987</v>
       </c>
-      <c r="K8" s="23" t="n">
+      <c r="K8" s="20" t="n">
         <v>37995</v>
       </c>
     </row>
@@ -5066,9 +5068,9 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:P16"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="32" customHeight="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
           <t>STUDYID</t>
@@ -5150,7 +5152,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
+    <row r="2" ht="96" customHeight="1">
       <c r="A2" s="9" t="inlineStr">
         <is>
           <t>Study Identifier</t>
@@ -5232,7 +5234,7 @@
         </is>
       </c>
     </row>
-    <row r="3">
+    <row r="3" ht="16" customHeight="1">
       <c r="A3" s="9" t="inlineStr">
         <is>
           <t>Char</t>
@@ -5364,891 +5366,891 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="24" t="inlineStr">
+    <row r="5" ht="48" customHeight="1">
+      <c r="A5" s="21" t="inlineStr">
         <is>
           <t>CDISCPILOT01</t>
         </is>
       </c>
-      <c r="B5" s="24" t="inlineStr">
+      <c r="B5" s="21" t="inlineStr">
         <is>
           <t>FA</t>
         </is>
       </c>
-      <c r="C5" s="24" t="inlineStr">
+      <c r="C5" s="21" t="inlineStr">
         <is>
           <t>CDISC001</t>
         </is>
       </c>
-      <c r="D5" s="24" t="n">
+      <c r="D5" s="21" t="n">
         <v>1</v>
       </c>
-      <c r="E5" s="24" t="inlineStr">
+      <c r="E5" s="21" t="inlineStr">
         <is>
           <t>CDISC001 - 1</t>
         </is>
       </c>
-      <c r="F5" s="24" t="inlineStr">
+      <c r="F5" s="21" t="inlineStr">
         <is>
           <t>OCCUR</t>
         </is>
       </c>
-      <c r="G5" s="24" t="inlineStr">
+      <c r="G5" s="21" t="inlineStr">
         <is>
           <t>Occurrence Indicator</t>
         </is>
       </c>
-      <c r="H5" s="24" t="inlineStr">
+      <c r="H5" s="21" t="inlineStr">
         <is>
           <t>ERYTHEMA</t>
         </is>
       </c>
-      <c r="I5" s="24" t="inlineStr">
+      <c r="I5" s="21" t="inlineStr">
         <is>
           <t>INJECTION SITE REACTION</t>
         </is>
       </c>
-      <c r="J5" s="24" t="inlineStr">
+      <c r="J5" s="21" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="K5" s="24" t="inlineStr">
+      <c r="K5" s="21" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="L5" s="24" t="inlineStr">
+      <c r="L5" s="21" t="inlineStr">
         <is>
           <t>ARM</t>
         </is>
       </c>
       <c r="M5" s="16" t="n"/>
-      <c r="N5" s="24" t="inlineStr">
+      <c r="N5" s="21" t="inlineStr">
         <is>
           <t>TREATMENT</t>
         </is>
       </c>
-      <c r="O5" s="24" t="inlineStr">
+      <c r="O5" s="21" t="inlineStr">
         <is>
           <t>2012-12-02</t>
         </is>
       </c>
-      <c r="P5" s="24" t="n">
+      <c r="P5" s="21" t="n">
         <v>3</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="24" t="inlineStr">
+    <row r="6" ht="48" customHeight="1">
+      <c r="A6" s="21" t="inlineStr">
         <is>
           <t>CDISCPILOT01</t>
         </is>
       </c>
-      <c r="B6" s="24" t="inlineStr">
+      <c r="B6" s="21" t="inlineStr">
         <is>
           <t>FA</t>
         </is>
       </c>
-      <c r="C6" s="24" t="inlineStr">
+      <c r="C6" s="21" t="inlineStr">
         <is>
           <t>CDISC001</t>
         </is>
       </c>
-      <c r="D6" s="24" t="n">
+      <c r="D6" s="21" t="n">
         <v>2</v>
       </c>
-      <c r="E6" s="24" t="inlineStr">
+      <c r="E6" s="21" t="inlineStr">
         <is>
           <t>CDISC001 - 1</t>
         </is>
       </c>
-      <c r="F6" s="24" t="inlineStr">
+      <c r="F6" s="21" t="inlineStr">
         <is>
           <t>SEV</t>
         </is>
       </c>
-      <c r="G6" s="24" t="inlineStr">
+      <c r="G6" s="21" t="inlineStr">
         <is>
           <t>Severity/Intensity</t>
         </is>
       </c>
-      <c r="H6" s="24" t="inlineStr">
+      <c r="H6" s="21" t="inlineStr">
         <is>
           <t>ERYTHEMA</t>
         </is>
       </c>
-      <c r="I6" s="24" t="inlineStr">
+      <c r="I6" s="21" t="inlineStr">
         <is>
           <t>INJECTION SITE REACTION</t>
         </is>
       </c>
-      <c r="J6" s="24" t="inlineStr">
+      <c r="J6" s="21" t="inlineStr">
         <is>
           <t>MODERATE</t>
         </is>
       </c>
-      <c r="K6" s="24" t="inlineStr">
+      <c r="K6" s="21" t="inlineStr">
         <is>
           <t>MODERATE</t>
         </is>
       </c>
-      <c r="L6" s="24" t="inlineStr">
+      <c r="L6" s="21" t="inlineStr">
         <is>
           <t>ARM</t>
         </is>
       </c>
       <c r="M6" s="16" t="n"/>
-      <c r="N6" s="24" t="inlineStr">
+      <c r="N6" s="21" t="inlineStr">
         <is>
           <t>TREATMENT</t>
         </is>
       </c>
-      <c r="O6" s="24" t="inlineStr">
+      <c r="O6" s="21" t="inlineStr">
         <is>
           <t>2012-12-02</t>
         </is>
       </c>
-      <c r="P6" s="24" t="n">
+      <c r="P6" s="21" t="n">
         <v>3</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="24" t="inlineStr">
+    <row r="7" ht="48" customHeight="1">
+      <c r="A7" s="21" t="inlineStr">
         <is>
           <t>CDISCPILOT01</t>
         </is>
       </c>
-      <c r="B7" s="24" t="inlineStr">
+      <c r="B7" s="21" t="inlineStr">
         <is>
           <t>FA</t>
         </is>
       </c>
-      <c r="C7" s="24" t="inlineStr">
+      <c r="C7" s="21" t="inlineStr">
         <is>
           <t>CDISC001</t>
         </is>
       </c>
-      <c r="D7" s="24" t="n">
+      <c r="D7" s="21" t="n">
         <v>3</v>
       </c>
-      <c r="E7" s="24" t="inlineStr">
+      <c r="E7" s="21" t="inlineStr">
         <is>
           <t>CDISC001 - 1</t>
         </is>
       </c>
-      <c r="F7" s="24" t="inlineStr">
+      <c r="F7" s="21" t="inlineStr">
         <is>
           <t>OCCUR</t>
         </is>
       </c>
-      <c r="G7" s="24" t="inlineStr">
+      <c r="G7" s="21" t="inlineStr">
         <is>
           <t>Occurrence Indicator</t>
         </is>
       </c>
-      <c r="H7" s="24" t="inlineStr">
+      <c r="H7" s="21" t="inlineStr">
         <is>
           <t>PAIN</t>
         </is>
       </c>
-      <c r="I7" s="24" t="inlineStr">
+      <c r="I7" s="21" t="inlineStr">
         <is>
           <t>INJECTION SITE REACTION</t>
         </is>
       </c>
-      <c r="J7" s="24" t="inlineStr">
+      <c r="J7" s="21" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="K7" s="24" t="inlineStr">
+      <c r="K7" s="21" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="L7" s="24" t="inlineStr">
+      <c r="L7" s="21" t="inlineStr">
         <is>
           <t>ARM</t>
         </is>
       </c>
       <c r="M7" s="16" t="n"/>
-      <c r="N7" s="24" t="inlineStr">
+      <c r="N7" s="21" t="inlineStr">
         <is>
           <t>TREATMENT</t>
         </is>
       </c>
-      <c r="O7" s="24" t="inlineStr">
+      <c r="O7" s="21" t="inlineStr">
         <is>
           <t>2012-12-02</t>
         </is>
       </c>
-      <c r="P7" s="24" t="n">
+      <c r="P7" s="21" t="n">
         <v>3</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="24" t="inlineStr">
+    <row r="8" ht="48" customHeight="1">
+      <c r="A8" s="21" t="inlineStr">
         <is>
           <t>CDISCPILOT01</t>
         </is>
       </c>
-      <c r="B8" s="24" t="inlineStr">
+      <c r="B8" s="21" t="inlineStr">
         <is>
           <t>FA</t>
         </is>
       </c>
-      <c r="C8" s="24" t="inlineStr">
+      <c r="C8" s="21" t="inlineStr">
         <is>
           <t>CDISC001</t>
         </is>
       </c>
-      <c r="D8" s="24" t="n">
+      <c r="D8" s="21" t="n">
         <v>4</v>
       </c>
-      <c r="E8" s="24" t="inlineStr">
+      <c r="E8" s="21" t="inlineStr">
         <is>
           <t>CDISC001 - 1</t>
         </is>
       </c>
-      <c r="F8" s="24" t="inlineStr">
+      <c r="F8" s="21" t="inlineStr">
         <is>
           <t>OCCUR</t>
         </is>
       </c>
-      <c r="G8" s="24" t="inlineStr">
+      <c r="G8" s="21" t="inlineStr">
         <is>
           <t>Occurrence Indicator</t>
         </is>
       </c>
-      <c r="H8" s="24" t="inlineStr">
+      <c r="H8" s="21" t="inlineStr">
         <is>
           <t>INDURATION</t>
         </is>
       </c>
-      <c r="I8" s="24" t="inlineStr">
+      <c r="I8" s="21" t="inlineStr">
         <is>
           <t>INJECTION SITE REACTION</t>
         </is>
       </c>
-      <c r="J8" s="24" t="inlineStr">
+      <c r="J8" s="21" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="K8" s="24" t="inlineStr">
+      <c r="K8" s="21" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="L8" s="24" t="inlineStr">
+      <c r="L8" s="21" t="inlineStr">
         <is>
           <t>ARM</t>
         </is>
       </c>
       <c r="M8" s="16" t="n"/>
-      <c r="N8" s="24" t="inlineStr">
+      <c r="N8" s="21" t="inlineStr">
         <is>
           <t>TREATMENT</t>
         </is>
       </c>
-      <c r="O8" s="24" t="inlineStr">
+      <c r="O8" s="21" t="inlineStr">
         <is>
           <t>2012-12-02</t>
         </is>
       </c>
-      <c r="P8" s="24" t="n">
+      <c r="P8" s="21" t="n">
         <v>3</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="24" t="inlineStr">
+    <row r="9" ht="48" customHeight="1">
+      <c r="A9" s="21" t="inlineStr">
         <is>
           <t>CDISCPILOT01</t>
         </is>
       </c>
-      <c r="B9" s="24" t="inlineStr">
+      <c r="B9" s="21" t="inlineStr">
         <is>
           <t>FA</t>
         </is>
       </c>
-      <c r="C9" s="24" t="inlineStr">
+      <c r="C9" s="21" t="inlineStr">
         <is>
           <t>CDISC001</t>
         </is>
       </c>
-      <c r="D9" s="24" t="n">
+      <c r="D9" s="21" t="n">
         <v>5</v>
       </c>
-      <c r="E9" s="24" t="inlineStr">
+      <c r="E9" s="21" t="inlineStr">
         <is>
           <t>CDISC001 - 1</t>
         </is>
       </c>
-      <c r="F9" s="24" t="inlineStr">
+      <c r="F9" s="21" t="inlineStr">
         <is>
           <t>OCCUR</t>
         </is>
       </c>
-      <c r="G9" s="24" t="inlineStr">
+      <c r="G9" s="21" t="inlineStr">
         <is>
           <t>Occurrence Indicator</t>
         </is>
       </c>
-      <c r="H9" s="24" t="inlineStr">
+      <c r="H9" s="21" t="inlineStr">
         <is>
           <t>PRURITIS</t>
         </is>
       </c>
-      <c r="I9" s="24" t="inlineStr">
+      <c r="I9" s="21" t="inlineStr">
         <is>
           <t>INJECTION SITE REACTION</t>
         </is>
       </c>
-      <c r="J9" s="24" t="inlineStr">
+      <c r="J9" s="21" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="K9" s="24" t="inlineStr">
+      <c r="K9" s="21" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="L9" s="24" t="inlineStr">
+      <c r="L9" s="21" t="inlineStr">
         <is>
           <t>ARM</t>
         </is>
       </c>
       <c r="M9" s="16" t="n"/>
-      <c r="N9" s="24" t="inlineStr">
+      <c r="N9" s="21" t="inlineStr">
         <is>
           <t>TREATMENT</t>
         </is>
       </c>
-      <c r="O9" s="24" t="inlineStr">
+      <c r="O9" s="21" t="inlineStr">
         <is>
           <t>2012-12-02</t>
         </is>
       </c>
-      <c r="P9" s="24" t="n">
+      <c r="P9" s="21" t="n">
         <v>3</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="24" t="inlineStr">
+    <row r="10" ht="48" customHeight="1">
+      <c r="A10" s="21" t="inlineStr">
         <is>
           <t>CDISCPILOT01</t>
         </is>
       </c>
-      <c r="B10" s="24" t="inlineStr">
+      <c r="B10" s="21" t="inlineStr">
         <is>
           <t>FA</t>
         </is>
       </c>
-      <c r="C10" s="24" t="inlineStr">
+      <c r="C10" s="21" t="inlineStr">
         <is>
           <t>CDISC001</t>
         </is>
       </c>
-      <c r="D10" s="24" t="n">
+      <c r="D10" s="21" t="n">
         <v>6</v>
       </c>
-      <c r="E10" s="24" t="inlineStr">
+      <c r="E10" s="21" t="inlineStr">
         <is>
           <t>CDISC001 - 1</t>
         </is>
       </c>
-      <c r="F10" s="24" t="inlineStr">
+      <c r="F10" s="21" t="inlineStr">
         <is>
           <t>OCCUR</t>
         </is>
       </c>
-      <c r="G10" s="24" t="inlineStr">
+      <c r="G10" s="21" t="inlineStr">
         <is>
           <t>Occurrence Indicator</t>
         </is>
       </c>
-      <c r="H10" s="24" t="inlineStr">
+      <c r="H10" s="21" t="inlineStr">
         <is>
           <t>EDEMA</t>
         </is>
       </c>
-      <c r="I10" s="24" t="inlineStr">
+      <c r="I10" s="21" t="inlineStr">
         <is>
           <t>INJECTION SITE REACTION</t>
         </is>
       </c>
-      <c r="J10" s="24" t="inlineStr">
+      <c r="J10" s="21" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="K10" s="24" t="inlineStr">
+      <c r="K10" s="21" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="L10" s="24" t="inlineStr">
+      <c r="L10" s="21" t="inlineStr">
         <is>
           <t>ARM</t>
         </is>
       </c>
       <c r="M10" s="16" t="n"/>
-      <c r="N10" s="24" t="inlineStr">
+      <c r="N10" s="21" t="inlineStr">
         <is>
           <t>TREATMENT</t>
         </is>
       </c>
-      <c r="O10" s="24" t="inlineStr">
+      <c r="O10" s="21" t="inlineStr">
         <is>
           <t>2012-12-02</t>
         </is>
       </c>
-      <c r="P10" s="24" t="n">
+      <c r="P10" s="21" t="n">
         <v>3</v>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="24" t="inlineStr">
+    <row r="11" ht="48" customHeight="1">
+      <c r="A11" s="21" t="inlineStr">
         <is>
           <t>CDISCPILOT01</t>
         </is>
       </c>
-      <c r="B11" s="24" t="inlineStr">
+      <c r="B11" s="21" t="inlineStr">
         <is>
           <t>FA</t>
         </is>
       </c>
-      <c r="C11" s="24" t="inlineStr">
+      <c r="C11" s="21" t="inlineStr">
         <is>
           <t>CDISC002</t>
         </is>
       </c>
-      <c r="D11" s="24" t="n">
+      <c r="D11" s="21" t="n">
         <v>1</v>
       </c>
-      <c r="E11" s="24" t="inlineStr">
+      <c r="E11" s="21" t="inlineStr">
         <is>
           <t>CDISC002 - 1</t>
         </is>
       </c>
-      <c r="F11" s="24" t="inlineStr">
+      <c r="F11" s="21" t="inlineStr">
         <is>
           <t>OCCUR</t>
         </is>
       </c>
-      <c r="G11" s="24" t="inlineStr">
+      <c r="G11" s="21" t="inlineStr">
         <is>
           <t>Occurrence Indicator</t>
         </is>
       </c>
-      <c r="H11" s="24" t="inlineStr">
+      <c r="H11" s="21" t="inlineStr">
         <is>
           <t>ERYTHEMA</t>
         </is>
       </c>
-      <c r="I11" s="24" t="inlineStr">
+      <c r="I11" s="21" t="inlineStr">
         <is>
           <t>INJECTION SITE REACTION</t>
         </is>
       </c>
-      <c r="J11" s="24" t="inlineStr">
+      <c r="J11" s="21" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="K11" s="24" t="inlineStr">
+      <c r="K11" s="21" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="L11" s="24" t="inlineStr">
+      <c r="L11" s="21" t="inlineStr">
         <is>
           <t>ARM</t>
         </is>
       </c>
       <c r="M11" s="16" t="n"/>
-      <c r="N11" s="24" t="inlineStr">
+      <c r="N11" s="21" t="inlineStr">
         <is>
           <t>TREATMENT</t>
         </is>
       </c>
-      <c r="O11" s="24" t="inlineStr">
+      <c r="O11" s="21" t="inlineStr">
         <is>
           <t>2012-11-16</t>
         </is>
       </c>
-      <c r="P11" s="24" t="n">
+      <c r="P11" s="21" t="n">
         <v>2</v>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="24" t="inlineStr">
+    <row r="12" ht="48" customHeight="1">
+      <c r="A12" s="21" t="inlineStr">
         <is>
           <t>CDISCPILOT01</t>
         </is>
       </c>
-      <c r="B12" s="24" t="inlineStr">
+      <c r="B12" s="21" t="inlineStr">
         <is>
           <t>FA</t>
         </is>
       </c>
-      <c r="C12" s="24" t="inlineStr">
+      <c r="C12" s="21" t="inlineStr">
         <is>
           <t>CDISC002</t>
         </is>
       </c>
-      <c r="D12" s="24" t="n">
+      <c r="D12" s="21" t="n">
         <v>2</v>
       </c>
-      <c r="E12" s="24" t="inlineStr">
+      <c r="E12" s="21" t="inlineStr">
         <is>
           <t>CDISC002 - 1</t>
         </is>
       </c>
-      <c r="F12" s="24" t="inlineStr">
+      <c r="F12" s="21" t="inlineStr">
         <is>
           <t>OCCUR</t>
         </is>
       </c>
-      <c r="G12" s="24" t="inlineStr">
+      <c r="G12" s="21" t="inlineStr">
         <is>
           <t>Occurrence Indicator</t>
         </is>
       </c>
-      <c r="H12" s="24" t="inlineStr">
+      <c r="H12" s="21" t="inlineStr">
         <is>
           <t>PAIN</t>
         </is>
       </c>
-      <c r="I12" s="24" t="inlineStr">
+      <c r="I12" s="21" t="inlineStr">
         <is>
           <t>INJECTION SITE REACTION</t>
         </is>
       </c>
-      <c r="J12" s="24" t="inlineStr">
+      <c r="J12" s="21" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="K12" s="24" t="inlineStr">
+      <c r="K12" s="21" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="L12" s="24" t="inlineStr">
+      <c r="L12" s="21" t="inlineStr">
         <is>
           <t>ARM</t>
         </is>
       </c>
       <c r="M12" s="16" t="n"/>
-      <c r="N12" s="24" t="inlineStr">
+      <c r="N12" s="21" t="inlineStr">
         <is>
           <t>TREATMENT</t>
         </is>
       </c>
-      <c r="O12" s="24" t="inlineStr">
+      <c r="O12" s="21" t="inlineStr">
         <is>
           <t>2012-11-16</t>
         </is>
       </c>
-      <c r="P12" s="24" t="n">
+      <c r="P12" s="21" t="n">
         <v>2</v>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="24" t="inlineStr">
+    <row r="13" ht="48" customHeight="1">
+      <c r="A13" s="21" t="inlineStr">
         <is>
           <t>CDISCPILOT01</t>
         </is>
       </c>
-      <c r="B13" s="24" t="inlineStr">
+      <c r="B13" s="21" t="inlineStr">
         <is>
           <t>FA</t>
         </is>
       </c>
-      <c r="C13" s="24" t="inlineStr">
+      <c r="C13" s="21" t="inlineStr">
         <is>
           <t>CDISC002</t>
         </is>
       </c>
-      <c r="D13" s="24" t="n">
+      <c r="D13" s="21" t="n">
         <v>3</v>
       </c>
-      <c r="E13" s="24" t="inlineStr">
+      <c r="E13" s="21" t="inlineStr">
         <is>
           <t>CDISC002 - 1</t>
         </is>
       </c>
-      <c r="F13" s="24" t="inlineStr">
+      <c r="F13" s="21" t="inlineStr">
         <is>
           <t>OCCUR</t>
         </is>
       </c>
-      <c r="G13" s="24" t="inlineStr">
+      <c r="G13" s="21" t="inlineStr">
         <is>
           <t>Occurrence Indicator</t>
         </is>
       </c>
-      <c r="H13" s="24" t="inlineStr">
+      <c r="H13" s="21" t="inlineStr">
         <is>
           <t>INDURATION</t>
         </is>
       </c>
-      <c r="I13" s="24" t="inlineStr">
+      <c r="I13" s="21" t="inlineStr">
         <is>
           <t>INJECTION SITE REACTION</t>
         </is>
       </c>
-      <c r="J13" s="24" t="inlineStr">
+      <c r="J13" s="21" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="K13" s="24" t="inlineStr">
+      <c r="K13" s="21" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="L13" s="24" t="inlineStr">
+      <c r="L13" s="21" t="inlineStr">
         <is>
           <t>ARM</t>
         </is>
       </c>
       <c r="M13" s="16" t="n"/>
-      <c r="N13" s="24" t="inlineStr">
+      <c r="N13" s="21" t="inlineStr">
         <is>
           <t>TREATMENT</t>
         </is>
       </c>
-      <c r="O13" s="24" t="inlineStr">
+      <c r="O13" s="21" t="inlineStr">
         <is>
           <t>2012-11-16</t>
         </is>
       </c>
-      <c r="P13" s="24" t="n">
+      <c r="P13" s="21" t="n">
         <v>2</v>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="24" t="inlineStr">
+    <row r="14" ht="48" customHeight="1">
+      <c r="A14" s="21" t="inlineStr">
         <is>
           <t>CDISCPILOT01</t>
         </is>
       </c>
-      <c r="B14" s="24" t="inlineStr">
+      <c r="B14" s="21" t="inlineStr">
         <is>
           <t>FA</t>
         </is>
       </c>
-      <c r="C14" s="24" t="inlineStr">
+      <c r="C14" s="21" t="inlineStr">
         <is>
           <t>CDISC002</t>
         </is>
       </c>
-      <c r="D14" s="24" t="n">
+      <c r="D14" s="21" t="n">
         <v>4</v>
       </c>
-      <c r="E14" s="24" t="inlineStr">
+      <c r="E14" s="21" t="inlineStr">
         <is>
           <t>CDISC002 - 1</t>
         </is>
       </c>
-      <c r="F14" s="24" t="inlineStr">
+      <c r="F14" s="21" t="inlineStr">
         <is>
           <t>OCCUR</t>
         </is>
       </c>
-      <c r="G14" s="24" t="inlineStr">
+      <c r="G14" s="21" t="inlineStr">
         <is>
           <t>Occurrence Indicator</t>
         </is>
       </c>
-      <c r="H14" s="24" t="inlineStr">
+      <c r="H14" s="21" t="inlineStr">
         <is>
           <t>PRURITIS</t>
         </is>
       </c>
-      <c r="I14" s="24" t="inlineStr">
+      <c r="I14" s="21" t="inlineStr">
         <is>
           <t>INJECTION SITE REACTION</t>
         </is>
       </c>
-      <c r="J14" s="24" t="inlineStr">
+      <c r="J14" s="21" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="K14" s="24" t="inlineStr">
+      <c r="K14" s="21" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="L14" s="24" t="inlineStr">
+      <c r="L14" s="21" t="inlineStr">
         <is>
           <t>ARM</t>
         </is>
       </c>
       <c r="M14" s="16" t="n"/>
-      <c r="N14" s="24" t="inlineStr">
+      <c r="N14" s="21" t="inlineStr">
         <is>
           <t>TREATMENT</t>
         </is>
       </c>
-      <c r="O14" s="24" t="inlineStr">
+      <c r="O14" s="21" t="inlineStr">
         <is>
           <t>2012-11-16</t>
         </is>
       </c>
-      <c r="P14" s="24" t="n">
+      <c r="P14" s="21" t="n">
         <v>2</v>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="24" t="inlineStr">
+    <row r="15" ht="48" customHeight="1">
+      <c r="A15" s="21" t="inlineStr">
         <is>
           <t>CDISCPILOT01</t>
         </is>
       </c>
-      <c r="B15" s="24" t="inlineStr">
+      <c r="B15" s="21" t="inlineStr">
         <is>
           <t>FA</t>
         </is>
       </c>
-      <c r="C15" s="24" t="inlineStr">
+      <c r="C15" s="21" t="inlineStr">
         <is>
           <t>CDISC002</t>
         </is>
       </c>
-      <c r="D15" s="24" t="n">
+      <c r="D15" s="21" t="n">
         <v>5</v>
       </c>
-      <c r="E15" s="24" t="inlineStr">
+      <c r="E15" s="21" t="inlineStr">
         <is>
           <t>CDISC002 - 1</t>
         </is>
       </c>
-      <c r="F15" s="24" t="inlineStr">
+      <c r="F15" s="21" t="inlineStr">
         <is>
           <t>SEV</t>
         </is>
       </c>
-      <c r="G15" s="24" t="inlineStr">
+      <c r="G15" s="21" t="inlineStr">
         <is>
           <t>Severity/Intensity</t>
         </is>
       </c>
-      <c r="H15" s="24" t="inlineStr">
+      <c r="H15" s="21" t="inlineStr">
         <is>
           <t>PRURITIS</t>
         </is>
       </c>
-      <c r="I15" s="24" t="inlineStr">
+      <c r="I15" s="21" t="inlineStr">
         <is>
           <t>INJECTION SITE REACTION</t>
         </is>
       </c>
-      <c r="J15" s="24" t="inlineStr">
+      <c r="J15" s="21" t="inlineStr">
         <is>
           <t>MILD</t>
         </is>
       </c>
-      <c r="K15" s="24" t="inlineStr">
+      <c r="K15" s="21" t="inlineStr">
         <is>
           <t>MILD</t>
         </is>
       </c>
-      <c r="L15" s="24" t="inlineStr">
+      <c r="L15" s="21" t="inlineStr">
         <is>
           <t>ARM</t>
         </is>
       </c>
       <c r="M15" s="16" t="n"/>
-      <c r="N15" s="24" t="inlineStr">
+      <c r="N15" s="21" t="inlineStr">
         <is>
           <t>TREATMENT</t>
         </is>
       </c>
-      <c r="O15" s="24" t="inlineStr">
+      <c r="O15" s="21" t="inlineStr">
         <is>
           <t>2012-11-16</t>
         </is>
       </c>
-      <c r="P15" s="24" t="n">
+      <c r="P15" s="21" t="n">
         <v>2</v>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="24" t="inlineStr">
+    <row r="16" ht="48" customHeight="1">
+      <c r="A16" s="21" t="inlineStr">
         <is>
           <t>CDISCPILOT01</t>
         </is>
       </c>
-      <c r="B16" s="24" t="inlineStr">
+      <c r="B16" s="21" t="inlineStr">
         <is>
           <t>FA</t>
         </is>
       </c>
-      <c r="C16" s="24" t="inlineStr">
+      <c r="C16" s="21" t="inlineStr">
         <is>
           <t>CDISC002</t>
         </is>
       </c>
-      <c r="D16" s="24" t="n">
+      <c r="D16" s="21" t="n">
         <v>6</v>
       </c>
-      <c r="E16" s="24" t="inlineStr">
+      <c r="E16" s="21" t="inlineStr">
         <is>
           <t>CDISC002 - 1</t>
         </is>
       </c>
-      <c r="F16" s="24" t="inlineStr">
+      <c r="F16" s="21" t="inlineStr">
         <is>
           <t>OCCUR</t>
         </is>
       </c>
-      <c r="G16" s="24" t="inlineStr">
+      <c r="G16" s="21" t="inlineStr">
         <is>
           <t>Occurrence Indicator</t>
         </is>
       </c>
-      <c r="H16" s="24" t="inlineStr">
+      <c r="H16" s="21" t="inlineStr">
         <is>
           <t>EDEMA</t>
         </is>
       </c>
-      <c r="I16" s="24" t="inlineStr">
+      <c r="I16" s="21" t="inlineStr">
         <is>
           <t>INJECTION SITE REACTION</t>
         </is>
       </c>
-      <c r="J16" s="24" t="inlineStr">
+      <c r="J16" s="21" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="K16" s="24" t="inlineStr">
+      <c r="K16" s="21" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="L16" s="24" t="inlineStr">
+      <c r="L16" s="21" t="inlineStr">
         <is>
           <t>ARM</t>
         </is>
       </c>
       <c r="M16" s="16" t="n"/>
-      <c r="N16" s="24" t="inlineStr">
+      <c r="N16" s="21" t="inlineStr">
         <is>
           <t>TREATMENT</t>
         </is>
       </c>
-      <c r="O16" s="24" t="inlineStr">
+      <c r="O16" s="21" t="inlineStr">
         <is>
           <t>2012-11-16</t>
         </is>
       </c>
-      <c r="P16" s="24" t="n">
+      <c r="P16" s="21" t="n">
         <v>2</v>
       </c>
     </row>

</xml_diff>